<commit_message>
Add agent loop, tools and CLI on Groq; working end-to-end
</commit_message>
<xml_diff>
--- a/data/synthetic/hr_headcount_comp.xlsx
+++ b/data/synthetic/hr_headcount_comp.xlsx
@@ -414,45 +414,105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F123"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>SYNTHETIC DATA - NOT REAL APPLE DATA - GENERATED FOR RBAC DEMO</t>
+          <t>fiscal_period</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>function</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>headcount</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>attrition_pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>open_roles</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>source_note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>10876</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F2" t="n">
+        <v>145</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>fiscal_period</t>
+          <t>FY2023</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>function</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>headcount</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>attrition_pct</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>open_roles</t>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4412</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F3" t="n">
+        <v>57</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
         </is>
       </c>
     </row>
@@ -469,17 +529,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>10876</v>
+        <v>11487</v>
       </c>
       <c r="E4" t="n">
-        <v>4.7</v>
+        <v>11.3</v>
       </c>
       <c r="F4" t="n">
-        <v>145</v>
+        <v>284</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -495,17 +560,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>4412</v>
+        <v>1824</v>
       </c>
       <c r="E5" t="n">
-        <v>5.8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>57</v>
+        <v>21</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -521,17 +591,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>11487</v>
+        <v>888</v>
       </c>
       <c r="E6" t="n">
-        <v>11.3</v>
+        <v>4.5</v>
       </c>
       <c r="F6" t="n">
-        <v>284</v>
+        <v>124</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -542,22 +617,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1824</v>
+        <v>8679</v>
       </c>
       <c r="E7" t="n">
-        <v>9.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>21</v>
+        <v>292</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -568,22 +648,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>888</v>
+        <v>3657</v>
       </c>
       <c r="E8" t="n">
-        <v>4.5</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
-        <v>124</v>
+        <v>284</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -599,17 +684,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8679</v>
+        <v>7273</v>
       </c>
       <c r="E9" t="n">
-        <v>9.800000000000001</v>
+        <v>5.8</v>
       </c>
       <c r="F9" t="n">
-        <v>292</v>
+        <v>147</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -625,17 +715,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3657</v>
+        <v>506</v>
       </c>
       <c r="E10" t="n">
-        <v>11</v>
+        <v>11.5</v>
       </c>
       <c r="F10" t="n">
-        <v>284</v>
+        <v>86</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -651,18 +746,23 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>7273</v>
+        <v>11838</v>
       </c>
       <c r="E11" t="n">
-        <v>5.8</v>
+        <v>7.9</v>
       </c>
       <c r="F11" t="n">
         <v>147</v>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -672,22 +772,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>506</v>
+        <v>2947</v>
       </c>
       <c r="E12" t="n">
-        <v>11.5</v>
+        <v>5.8</v>
       </c>
       <c r="F12" t="n">
-        <v>86</v>
+        <v>177</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -698,22 +803,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>11838</v>
+        <v>2074</v>
       </c>
       <c r="E13" t="n">
-        <v>7.9</v>
+        <v>4.5</v>
       </c>
       <c r="F13" t="n">
-        <v>147</v>
+        <v>54</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -729,17 +839,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2947</v>
+        <v>6281</v>
       </c>
       <c r="E14" t="n">
-        <v>5.8</v>
+        <v>12.4</v>
       </c>
       <c r="F14" t="n">
-        <v>177</v>
+        <v>140</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -755,17 +870,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2074</v>
+        <v>1111</v>
       </c>
       <c r="E15" t="n">
-        <v>4.5</v>
+        <v>11.2</v>
       </c>
       <c r="F15" t="n">
-        <v>54</v>
+        <v>279</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -781,17 +901,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6281</v>
+        <v>2445</v>
       </c>
       <c r="E16" t="n">
-        <v>12.4</v>
+        <v>13.7</v>
       </c>
       <c r="F16" t="n">
-        <v>140</v>
+        <v>198</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -802,22 +927,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1111</v>
+        <v>1691</v>
       </c>
       <c r="E17" t="n">
-        <v>11.2</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>279</v>
+        <v>190</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -828,22 +958,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2445</v>
+        <v>9859</v>
       </c>
       <c r="E18" t="n">
-        <v>13.7</v>
+        <v>5.5</v>
       </c>
       <c r="F18" t="n">
-        <v>198</v>
+        <v>40</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -859,17 +994,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1691</v>
+        <v>1150</v>
       </c>
       <c r="E19" t="n">
-        <v>9.300000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="F19" t="n">
-        <v>190</v>
+        <v>153</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -885,17 +1025,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>9859</v>
+        <v>1707</v>
       </c>
       <c r="E20" t="n">
-        <v>5.5</v>
+        <v>12.5</v>
       </c>
       <c r="F20" t="n">
-        <v>40</v>
+        <v>56</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -911,17 +1056,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1150</v>
+        <v>6627</v>
       </c>
       <c r="E21" t="n">
-        <v>10.4</v>
+        <v>6.4</v>
       </c>
       <c r="F21" t="n">
-        <v>153</v>
+        <v>191</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -932,22 +1082,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1707</v>
+        <v>3064</v>
       </c>
       <c r="E22" t="n">
-        <v>12.5</v>
+        <v>7.4</v>
       </c>
       <c r="F22" t="n">
-        <v>56</v>
+        <v>112</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -958,22 +1113,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6627</v>
+        <v>11380</v>
       </c>
       <c r="E23" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="F23" t="n">
-        <v>191</v>
+        <v>41</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -989,17 +1149,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3064</v>
+        <v>10380</v>
       </c>
       <c r="E24" t="n">
-        <v>7.4</v>
+        <v>10.2</v>
       </c>
       <c r="F24" t="n">
-        <v>112</v>
+        <v>278</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1015,17 +1180,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>11380</v>
+        <v>4410</v>
       </c>
       <c r="E25" t="n">
-        <v>6.3</v>
+        <v>5.2</v>
       </c>
       <c r="F25" t="n">
-        <v>41</v>
+        <v>199</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1041,17 +1211,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>10380</v>
+        <v>4822</v>
       </c>
       <c r="E26" t="n">
-        <v>10.2</v>
+        <v>13.9</v>
       </c>
       <c r="F26" t="n">
-        <v>278</v>
+        <v>290</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -1062,22 +1237,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>4410</v>
+        <v>3998</v>
       </c>
       <c r="E27" t="n">
-        <v>5.2</v>
+        <v>10.7</v>
       </c>
       <c r="F27" t="n">
-        <v>199</v>
+        <v>33</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1088,22 +1268,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4822</v>
+        <v>4152</v>
       </c>
       <c r="E28" t="n">
-        <v>13.9</v>
+        <v>12.1</v>
       </c>
       <c r="F28" t="n">
-        <v>290</v>
+        <v>166</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1119,17 +1304,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3998</v>
+        <v>6972</v>
       </c>
       <c r="E29" t="n">
-        <v>10.7</v>
+        <v>6.3</v>
       </c>
       <c r="F29" t="n">
-        <v>33</v>
+        <v>113</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1145,18 +1335,23 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>4152</v>
+        <v>9692</v>
       </c>
       <c r="E30" t="n">
-        <v>12.1</v>
+        <v>12.7</v>
       </c>
       <c r="F30" t="n">
         <v>166</v>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1171,17 +1366,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>6972</v>
+        <v>3883</v>
       </c>
       <c r="E31" t="n">
-        <v>6.3</v>
+        <v>10.4</v>
       </c>
       <c r="F31" t="n">
-        <v>113</v>
+        <v>207</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -1192,22 +1392,27 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>9692</v>
+        <v>10932</v>
       </c>
       <c r="E32" t="n">
-        <v>12.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F32" t="n">
-        <v>166</v>
+        <v>140</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1218,22 +1423,27 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3883</v>
+        <v>2687</v>
       </c>
       <c r="E33" t="n">
-        <v>10.4</v>
+        <v>6.1</v>
       </c>
       <c r="F33" t="n">
-        <v>207</v>
+        <v>292</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1249,17 +1459,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>10932</v>
+        <v>9230</v>
       </c>
       <c r="E34" t="n">
-        <v>8.300000000000001</v>
+        <v>6.3</v>
       </c>
       <c r="F34" t="n">
-        <v>140</v>
+        <v>224</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1275,17 +1490,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>2687</v>
+        <v>9960</v>
       </c>
       <c r="E35" t="n">
-        <v>6.1</v>
+        <v>7.7</v>
       </c>
       <c r="F35" t="n">
-        <v>292</v>
+        <v>117</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -1301,17 +1521,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>9230</v>
+        <v>2666</v>
       </c>
       <c r="E36" t="n">
-        <v>6.3</v>
+        <v>8.9</v>
       </c>
       <c r="F36" t="n">
-        <v>224</v>
+        <v>51</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1322,22 +1547,27 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>9960</v>
+        <v>1171</v>
       </c>
       <c r="E37" t="n">
-        <v>7.7</v>
+        <v>12.5</v>
       </c>
       <c r="F37" t="n">
-        <v>117</v>
+        <v>83</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1348,22 +1578,27 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2666</v>
+        <v>10680</v>
       </c>
       <c r="E38" t="n">
-        <v>8.9</v>
+        <v>5.2</v>
       </c>
       <c r="F38" t="n">
-        <v>51</v>
+        <v>221</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1379,17 +1614,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1171</v>
+        <v>10171</v>
       </c>
       <c r="E39" t="n">
-        <v>12.5</v>
+        <v>4.2</v>
       </c>
       <c r="F39" t="n">
-        <v>83</v>
+        <v>200</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -1405,17 +1645,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>10680</v>
+        <v>10163</v>
       </c>
       <c r="E40" t="n">
-        <v>5.2</v>
+        <v>14</v>
       </c>
       <c r="F40" t="n">
-        <v>221</v>
+        <v>275</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -1431,69 +1676,84 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>10171</v>
+        <v>4519</v>
       </c>
       <c r="E41" t="n">
-        <v>4.2</v>
+        <v>13.7</v>
       </c>
       <c r="F41" t="n">
-        <v>200</v>
+        <v>10</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>FY2023</t>
+          <t>FY2024</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>10163</v>
+        <v>11545</v>
       </c>
       <c r="E42" t="n">
-        <v>14</v>
+        <v>11.1</v>
       </c>
       <c r="F42" t="n">
-        <v>275</v>
+        <v>279</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FY2023</t>
+          <t>FY2024</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>4519</v>
+        <v>4771</v>
       </c>
       <c r="E43" t="n">
-        <v>13.7</v>
+        <v>11.6</v>
       </c>
       <c r="F43" t="n">
-        <v>10</v>
+        <v>179</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -1509,17 +1769,22 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>11545</v>
+        <v>2227</v>
       </c>
       <c r="E44" t="n">
-        <v>11.1</v>
+        <v>6.6</v>
       </c>
       <c r="F44" t="n">
-        <v>279</v>
+        <v>85</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -1535,17 +1800,22 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>4771</v>
+        <v>7833</v>
       </c>
       <c r="E45" t="n">
-        <v>11.6</v>
+        <v>3.5</v>
       </c>
       <c r="F45" t="n">
-        <v>179</v>
+        <v>139</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -1561,17 +1831,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2227</v>
+        <v>8601</v>
       </c>
       <c r="E46" t="n">
-        <v>6.6</v>
+        <v>11.5</v>
       </c>
       <c r="F46" t="n">
-        <v>85</v>
+        <v>264</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -1582,22 +1857,27 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>7833</v>
+        <v>2143</v>
       </c>
       <c r="E47" t="n">
-        <v>3.5</v>
+        <v>12.6</v>
       </c>
       <c r="F47" t="n">
-        <v>139</v>
+        <v>157</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -1608,22 +1888,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>8601</v>
+        <v>10868</v>
       </c>
       <c r="E48" t="n">
-        <v>11.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F48" t="n">
-        <v>264</v>
+        <v>106</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -1639,17 +1924,22 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>2143</v>
+        <v>2904</v>
       </c>
       <c r="E49" t="n">
-        <v>12.6</v>
+        <v>7.4</v>
       </c>
       <c r="F49" t="n">
-        <v>157</v>
+        <v>87</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -1665,17 +1955,22 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>10868</v>
+        <v>9237</v>
       </c>
       <c r="E50" t="n">
-        <v>8.800000000000001</v>
+        <v>13.5</v>
       </c>
       <c r="F50" t="n">
-        <v>106</v>
+        <v>276</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -1691,17 +1986,22 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2904</v>
+        <v>409</v>
       </c>
       <c r="E51" t="n">
-        <v>7.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F51" t="n">
-        <v>87</v>
+        <v>255</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -1712,22 +2012,27 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>9237</v>
+        <v>719</v>
       </c>
       <c r="E52" t="n">
-        <v>13.5</v>
+        <v>4.7</v>
       </c>
       <c r="F52" t="n">
-        <v>276</v>
+        <v>190</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -1738,22 +2043,27 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>409</v>
+        <v>5438</v>
       </c>
       <c r="E53" t="n">
-        <v>9.800000000000001</v>
+        <v>6</v>
       </c>
       <c r="F53" t="n">
-        <v>255</v>
+        <v>128</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -1769,17 +2079,22 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>719</v>
+        <v>9695</v>
       </c>
       <c r="E54" t="n">
-        <v>4.7</v>
+        <v>13.4</v>
       </c>
       <c r="F54" t="n">
-        <v>190</v>
+        <v>48</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -1795,17 +2110,22 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>5438</v>
+        <v>8362</v>
       </c>
       <c r="E55" t="n">
-        <v>6</v>
+        <v>12.1</v>
       </c>
       <c r="F55" t="n">
-        <v>128</v>
+        <v>277</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -1821,17 +2141,22 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>9695</v>
+        <v>2460</v>
       </c>
       <c r="E56" t="n">
-        <v>13.4</v>
+        <v>4.8</v>
       </c>
       <c r="F56" t="n">
-        <v>48</v>
+        <v>248</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -1842,22 +2167,27 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>8362</v>
+        <v>9407</v>
       </c>
       <c r="E57" t="n">
-        <v>12.1</v>
+        <v>5.2</v>
       </c>
       <c r="F57" t="n">
-        <v>277</v>
+        <v>275</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -1868,22 +2198,27 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>2460</v>
+        <v>10338</v>
       </c>
       <c r="E58" t="n">
-        <v>4.8</v>
+        <v>7.9</v>
       </c>
       <c r="F58" t="n">
-        <v>248</v>
+        <v>113</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -1899,17 +2234,22 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>9407</v>
+        <v>9235</v>
       </c>
       <c r="E59" t="n">
-        <v>5.2</v>
+        <v>11.4</v>
       </c>
       <c r="F59" t="n">
-        <v>275</v>
+        <v>107</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -1925,17 +2265,22 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>10338</v>
+        <v>5507</v>
       </c>
       <c r="E60" t="n">
-        <v>7.9</v>
+        <v>7.7</v>
       </c>
       <c r="F60" t="n">
-        <v>113</v>
+        <v>196</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -1951,17 +2296,22 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>9235</v>
+        <v>7577</v>
       </c>
       <c r="E61" t="n">
-        <v>11.4</v>
+        <v>12.9</v>
       </c>
       <c r="F61" t="n">
-        <v>107</v>
+        <v>236</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -1972,22 +2322,27 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>5507</v>
+        <v>2382</v>
       </c>
       <c r="E62" t="n">
-        <v>7.7</v>
+        <v>6.1</v>
       </c>
       <c r="F62" t="n">
-        <v>196</v>
+        <v>37</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -1998,22 +2353,27 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>7577</v>
+        <v>5939</v>
       </c>
       <c r="E63" t="n">
-        <v>12.9</v>
+        <v>3.7</v>
       </c>
       <c r="F63" t="n">
-        <v>236</v>
+        <v>288</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -2029,17 +2389,22 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>2382</v>
+        <v>4170</v>
       </c>
       <c r="E64" t="n">
-        <v>6.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F64" t="n">
-        <v>37</v>
+        <v>8</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -2055,17 +2420,22 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>5939</v>
+        <v>1563</v>
       </c>
       <c r="E65" t="n">
-        <v>3.7</v>
+        <v>10.9</v>
       </c>
       <c r="F65" t="n">
-        <v>288</v>
+        <v>35</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -2081,17 +2451,22 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>4170</v>
+        <v>4150</v>
       </c>
       <c r="E66" t="n">
-        <v>9.699999999999999</v>
+        <v>4.2</v>
       </c>
       <c r="F66" t="n">
-        <v>8</v>
+        <v>21</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -2102,22 +2477,27 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1563</v>
+        <v>5813</v>
       </c>
       <c r="E67" t="n">
-        <v>10.9</v>
+        <v>4.2</v>
       </c>
       <c r="F67" t="n">
-        <v>35</v>
+        <v>126</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -2128,22 +2508,27 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>4150</v>
+        <v>4962</v>
       </c>
       <c r="E68" t="n">
-        <v>4.2</v>
+        <v>10.5</v>
       </c>
       <c r="F68" t="n">
-        <v>21</v>
+        <v>114</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -2159,17 +2544,22 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>5813</v>
+        <v>9234</v>
       </c>
       <c r="E69" t="n">
-        <v>4.2</v>
+        <v>4.9</v>
       </c>
       <c r="F69" t="n">
-        <v>126</v>
+        <v>297</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -2185,17 +2575,22 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>4962</v>
+        <v>9840</v>
       </c>
       <c r="E70" t="n">
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="F70" t="n">
-        <v>114</v>
+        <v>247</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -2211,17 +2606,22 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>9234</v>
+        <v>7069</v>
       </c>
       <c r="E71" t="n">
-        <v>4.9</v>
+        <v>5.5</v>
       </c>
       <c r="F71" t="n">
-        <v>297</v>
+        <v>54</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -2232,22 +2632,27 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>9840</v>
+        <v>11196</v>
       </c>
       <c r="E72" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="F72" t="n">
-        <v>247</v>
+        <v>221</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -2258,22 +2663,27 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>7069</v>
+        <v>7135</v>
       </c>
       <c r="E73" t="n">
-        <v>5.5</v>
+        <v>8.4</v>
       </c>
       <c r="F73" t="n">
-        <v>54</v>
+        <v>32</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -2289,17 +2699,22 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>11196</v>
+        <v>11432</v>
       </c>
       <c r="E74" t="n">
-        <v>8</v>
+        <v>10.4</v>
       </c>
       <c r="F74" t="n">
-        <v>221</v>
+        <v>55</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -2315,17 +2730,22 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>7135</v>
+        <v>1393</v>
       </c>
       <c r="E75" t="n">
-        <v>8.4</v>
+        <v>7.7</v>
       </c>
       <c r="F75" t="n">
-        <v>32</v>
+        <v>178</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -2341,17 +2761,22 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>11432</v>
+        <v>2190</v>
       </c>
       <c r="E76" t="n">
-        <v>10.4</v>
+        <v>6.1</v>
       </c>
       <c r="F76" t="n">
-        <v>55</v>
+        <v>102</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -2362,22 +2787,27 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1393</v>
+        <v>9186</v>
       </c>
       <c r="E77" t="n">
-        <v>7.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F77" t="n">
-        <v>178</v>
+        <v>221</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -2388,22 +2818,27 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>2190</v>
+        <v>3406</v>
       </c>
       <c r="E78" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="F78" t="n">
-        <v>102</v>
+        <v>132</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -2419,17 +2854,22 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>9186</v>
+        <v>1635</v>
       </c>
       <c r="E79" t="n">
         <v>8.199999999999999</v>
       </c>
       <c r="F79" t="n">
-        <v>221</v>
+        <v>286</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -2445,17 +2885,22 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>3406</v>
+        <v>2004</v>
       </c>
       <c r="E80" t="n">
-        <v>6.4</v>
+        <v>4</v>
       </c>
       <c r="F80" t="n">
-        <v>132</v>
+        <v>281</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -2471,69 +2916,84 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1635</v>
+        <v>641</v>
       </c>
       <c r="E81" t="n">
-        <v>8.199999999999999</v>
+        <v>13.7</v>
       </c>
       <c r="F81" t="n">
-        <v>286</v>
+        <v>126</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2025</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>2004</v>
+        <v>3124</v>
       </c>
       <c r="E82" t="n">
-        <v>4</v>
+        <v>7.8</v>
       </c>
       <c r="F82" t="n">
-        <v>281</v>
+        <v>251</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2025</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>641</v>
+        <v>3902</v>
       </c>
       <c r="E83" t="n">
-        <v>13.7</v>
+        <v>12.6</v>
       </c>
       <c r="F83" t="n">
-        <v>126</v>
+        <v>35</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -2549,17 +3009,22 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>3124</v>
+        <v>3097</v>
       </c>
       <c r="E84" t="n">
-        <v>7.8</v>
+        <v>7.5</v>
       </c>
       <c r="F84" t="n">
-        <v>251</v>
+        <v>204</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -2575,17 +3040,22 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>3902</v>
+        <v>4745</v>
       </c>
       <c r="E85" t="n">
-        <v>12.6</v>
+        <v>13.2</v>
       </c>
       <c r="F85" t="n">
-        <v>35</v>
+        <v>237</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -2601,17 +3071,22 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>3097</v>
+        <v>5073</v>
       </c>
       <c r="E86" t="n">
-        <v>7.5</v>
+        <v>7.9</v>
       </c>
       <c r="F86" t="n">
-        <v>204</v>
+        <v>289</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -2622,22 +3097,27 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>4745</v>
+        <v>11244</v>
       </c>
       <c r="E87" t="n">
-        <v>13.2</v>
+        <v>11</v>
       </c>
       <c r="F87" t="n">
-        <v>237</v>
+        <v>84</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="88">
@@ -2648,22 +3128,27 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>5073</v>
+        <v>3511</v>
       </c>
       <c r="E88" t="n">
-        <v>7.9</v>
+        <v>6.6</v>
       </c>
       <c r="F88" t="n">
-        <v>289</v>
+        <v>34</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -2679,17 +3164,22 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>11244</v>
+        <v>9889</v>
       </c>
       <c r="E89" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="F89" t="n">
-        <v>84</v>
+        <v>36</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -2705,17 +3195,22 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>3511</v>
+        <v>5538</v>
       </c>
       <c r="E90" t="n">
-        <v>6.6</v>
+        <v>4.1</v>
       </c>
       <c r="F90" t="n">
-        <v>34</v>
+        <v>249</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -2731,17 +3226,22 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>9889</v>
+        <v>8638</v>
       </c>
       <c r="E91" t="n">
-        <v>11.2</v>
+        <v>13.2</v>
       </c>
       <c r="F91" t="n">
-        <v>36</v>
+        <v>276</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="92">
@@ -2752,22 +3252,27 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>5538</v>
+        <v>2979</v>
       </c>
       <c r="E92" t="n">
         <v>4.1</v>
       </c>
       <c r="F92" t="n">
-        <v>249</v>
+        <v>265</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="93">
@@ -2778,22 +3283,27 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>8638</v>
+        <v>1712</v>
       </c>
       <c r="E93" t="n">
-        <v>13.2</v>
+        <v>12.4</v>
       </c>
       <c r="F93" t="n">
-        <v>276</v>
+        <v>40</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="94">
@@ -2809,17 +3319,22 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>2979</v>
+        <v>10149</v>
       </c>
       <c r="E94" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="F94" t="n">
-        <v>265</v>
+        <v>125</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="95">
@@ -2835,17 +3350,22 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>1712</v>
+        <v>7015</v>
       </c>
       <c r="E95" t="n">
-        <v>12.4</v>
+        <v>4.8</v>
       </c>
       <c r="F95" t="n">
-        <v>40</v>
+        <v>296</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -2861,17 +3381,22 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>10149</v>
+        <v>4433</v>
       </c>
       <c r="E96" t="n">
-        <v>4.2</v>
+        <v>9.6</v>
       </c>
       <c r="F96" t="n">
-        <v>125</v>
+        <v>25</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -2882,22 +3407,27 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>7015</v>
+        <v>10547</v>
       </c>
       <c r="E97" t="n">
-        <v>4.8</v>
+        <v>4.4</v>
       </c>
       <c r="F97" t="n">
-        <v>296</v>
+        <v>294</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="98">
@@ -2908,22 +3438,27 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>4433</v>
+        <v>8965</v>
       </c>
       <c r="E98" t="n">
-        <v>9.6</v>
+        <v>6.8</v>
       </c>
       <c r="F98" t="n">
-        <v>25</v>
+        <v>138</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -2939,17 +3474,22 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>10547</v>
+        <v>3746</v>
       </c>
       <c r="E99" t="n">
-        <v>4.4</v>
+        <v>10.5</v>
       </c>
       <c r="F99" t="n">
-        <v>294</v>
+        <v>165</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -2965,17 +3505,22 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>8965</v>
+        <v>4310</v>
       </c>
       <c r="E100" t="n">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="F100" t="n">
-        <v>138</v>
+        <v>72</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -2991,17 +3536,22 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>3746</v>
+        <v>11404</v>
       </c>
       <c r="E101" t="n">
-        <v>10.5</v>
+        <v>10.3</v>
       </c>
       <c r="F101" t="n">
-        <v>165</v>
+        <v>239</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="102">
@@ -3012,22 +3562,27 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>4310</v>
+        <v>5580</v>
       </c>
       <c r="E102" t="n">
-        <v>6.3</v>
+        <v>13.3</v>
       </c>
       <c r="F102" t="n">
-        <v>72</v>
+        <v>42</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="103">
@@ -3038,22 +3593,27 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>11404</v>
+        <v>552</v>
       </c>
       <c r="E103" t="n">
-        <v>10.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F103" t="n">
-        <v>239</v>
+        <v>293</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="104">
@@ -3069,17 +3629,22 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>5580</v>
+        <v>2038</v>
       </c>
       <c r="E104" t="n">
-        <v>13.3</v>
+        <v>4.3</v>
       </c>
       <c r="F104" t="n">
-        <v>42</v>
+        <v>114</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="105">
@@ -3095,17 +3660,22 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>552</v>
+        <v>8688</v>
       </c>
       <c r="E105" t="n">
-        <v>8.300000000000001</v>
+        <v>6.3</v>
       </c>
       <c r="F105" t="n">
-        <v>293</v>
+        <v>183</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -3121,17 +3691,22 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>2038</v>
+        <v>1527</v>
       </c>
       <c r="E106" t="n">
-        <v>4.3</v>
+        <v>12.7</v>
       </c>
       <c r="F106" t="n">
-        <v>114</v>
+        <v>194</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="107">
@@ -3142,22 +3717,27 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>8688</v>
+        <v>5069</v>
       </c>
       <c r="E107" t="n">
-        <v>6.3</v>
+        <v>5.2</v>
       </c>
       <c r="F107" t="n">
-        <v>183</v>
+        <v>283</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="108">
@@ -3168,22 +3748,27 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>1527</v>
+        <v>11926</v>
       </c>
       <c r="E108" t="n">
-        <v>12.7</v>
+        <v>6.7</v>
       </c>
       <c r="F108" t="n">
-        <v>194</v>
+        <v>275</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="109">
@@ -3199,17 +3784,22 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>5069</v>
+        <v>528</v>
       </c>
       <c r="E109" t="n">
-        <v>5.2</v>
+        <v>10.5</v>
       </c>
       <c r="F109" t="n">
-        <v>283</v>
+        <v>288</v>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="110">
@@ -3225,17 +3815,22 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>11926</v>
+        <v>5305</v>
       </c>
       <c r="E110" t="n">
-        <v>6.7</v>
+        <v>13.3</v>
       </c>
       <c r="F110" t="n">
-        <v>275</v>
+        <v>58</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="111">
@@ -3251,17 +3846,22 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>528</v>
+        <v>2600</v>
       </c>
       <c r="E111" t="n">
-        <v>10.5</v>
+        <v>6.3</v>
       </c>
       <c r="F111" t="n">
-        <v>288</v>
+        <v>59</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="112">
@@ -3272,22 +3872,27 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>5305</v>
+        <v>9464</v>
       </c>
       <c r="E112" t="n">
-        <v>13.3</v>
+        <v>5.1</v>
       </c>
       <c r="F112" t="n">
-        <v>58</v>
+        <v>149</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="113">
@@ -3298,22 +3903,27 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>2600</v>
+        <v>10309</v>
       </c>
       <c r="E113" t="n">
-        <v>6.3</v>
+        <v>5.7</v>
       </c>
       <c r="F113" t="n">
-        <v>59</v>
+        <v>180</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="114">
@@ -3329,17 +3939,22 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>9464</v>
+        <v>3735</v>
       </c>
       <c r="E114" t="n">
-        <v>5.1</v>
+        <v>10.7</v>
       </c>
       <c r="F114" t="n">
-        <v>149</v>
+        <v>140</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="115">
@@ -3355,17 +3970,22 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>10309</v>
+        <v>8680</v>
       </c>
       <c r="E115" t="n">
-        <v>5.7</v>
+        <v>8.6</v>
       </c>
       <c r="F115" t="n">
-        <v>180</v>
+        <v>31</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="116">
@@ -3381,17 +4001,22 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>3735</v>
+        <v>1912</v>
       </c>
       <c r="E116" t="n">
-        <v>10.7</v>
+        <v>10.2</v>
       </c>
       <c r="F116" t="n">
-        <v>140</v>
+        <v>146</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="117">
@@ -3402,22 +4027,27 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Americas</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>8680</v>
+        <v>1122</v>
       </c>
       <c r="E117" t="n">
-        <v>8.6</v>
+        <v>3.5</v>
       </c>
       <c r="F117" t="n">
-        <v>31</v>
+        <v>71</v>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="118">
@@ -3428,22 +4058,27 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Rest of Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>1912</v>
+        <v>10838</v>
       </c>
       <c r="E118" t="n">
-        <v>10.2</v>
+        <v>13.8</v>
       </c>
       <c r="F118" t="n">
-        <v>146</v>
+        <v>87</v>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="119">
@@ -3459,17 +4094,22 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Greater China</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>1122</v>
+        <v>7639</v>
       </c>
       <c r="E119" t="n">
-        <v>3.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F119" t="n">
-        <v>71</v>
+        <v>223</v>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -3485,17 +4125,22 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>10838</v>
+        <v>9589</v>
       </c>
       <c r="E120" t="n">
-        <v>13.8</v>
+        <v>3.6</v>
       </c>
       <c r="F120" t="n">
-        <v>87</v>
+        <v>43</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="121">
@@ -3511,69 +4156,22 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Greater China</t>
+          <t>Rest of Asia Pacific</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>7639</v>
+        <v>11721</v>
       </c>
       <c r="E121" t="n">
-        <v>9.300000000000001</v>
+        <v>13</v>
       </c>
       <c r="F121" t="n">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>FY2025</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D122" t="n">
-        <v>9589</v>
-      </c>
-      <c r="E122" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="F122" t="n">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>FY2025</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>Rest of Asia Pacific</t>
-        </is>
-      </c>
-      <c r="D123" t="n">
-        <v>11721</v>
-      </c>
-      <c r="E123" t="n">
-        <v>13</v>
-      </c>
-      <c r="F123" t="n">
         <v>284</v>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3587,50 +4185,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>SYNTHETIC DATA - NOT REAL APPLE DATA - GENERATED FOR RBAC DEMO</t>
+          <t>fiscal_period</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>function</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>band_min_usd</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>band_median_usd</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>band_max_usd</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>avg_equity_grant_usd</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>bonus_target_pct</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>source_note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>99000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>133650</v>
+      </c>
+      <c r="E2" t="n">
+        <v>188100</v>
+      </c>
+      <c r="F2" t="n">
+        <v>114000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>fiscal_period</t>
+          <t>FY2023</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>function</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>band_min_usd</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>band_median_usd</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>band_max_usd</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>avg_equity_grant_usd</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>bonus_target_pct</t>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>165000</v>
+      </c>
+      <c r="D3" t="n">
+        <v>222750</v>
+      </c>
+      <c r="E3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="F3" t="n">
+        <v>57000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>25</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
         </is>
       </c>
     </row>
@@ -3642,23 +4302,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>99000</v>
+        <v>111000</v>
       </c>
       <c r="D4" t="n">
-        <v>133650</v>
+        <v>149850</v>
       </c>
       <c r="E4" t="n">
-        <v>188100</v>
+        <v>210900</v>
       </c>
       <c r="F4" t="n">
-        <v>114000</v>
+        <v>30000</v>
       </c>
       <c r="G4" t="n">
-        <v>30</v>
+        <v>20</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -3669,23 +4334,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>165000</v>
+        <v>141000</v>
       </c>
       <c r="D5" t="n">
-        <v>222750</v>
+        <v>190350</v>
       </c>
       <c r="E5" t="n">
-        <v>313500</v>
+        <v>267900</v>
       </c>
       <c r="F5" t="n">
-        <v>57000</v>
+        <v>30000</v>
       </c>
       <c r="G5" t="n">
-        <v>25</v>
+        <v>20</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -3696,23 +4366,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>111000</v>
+        <v>121000</v>
       </c>
       <c r="D6" t="n">
-        <v>149850</v>
+        <v>163350</v>
       </c>
       <c r="E6" t="n">
-        <v>210900</v>
+        <v>229900</v>
       </c>
       <c r="F6" t="n">
-        <v>30000</v>
+        <v>83000</v>
       </c>
       <c r="G6" t="n">
-        <v>20</v>
+        <v>10</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -3723,23 +4398,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>141000</v>
+        <v>140000</v>
       </c>
       <c r="D7" t="n">
-        <v>190350</v>
+        <v>189000</v>
       </c>
       <c r="E7" t="n">
-        <v>267900</v>
+        <v>266000</v>
       </c>
       <c r="F7" t="n">
-        <v>30000</v>
+        <v>163000</v>
       </c>
       <c r="G7" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -3750,23 +4430,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>121000</v>
+        <v>174000</v>
       </c>
       <c r="D8" t="n">
-        <v>163350</v>
+        <v>234900</v>
       </c>
       <c r="E8" t="n">
-        <v>229900</v>
+        <v>330600</v>
       </c>
       <c r="F8" t="n">
-        <v>83000</v>
+        <v>59000</v>
       </c>
       <c r="G8" t="n">
-        <v>10</v>
+        <v>15</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -3777,77 +4462,92 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>140000</v>
+        <v>205000</v>
       </c>
       <c r="D9" t="n">
-        <v>189000</v>
+        <v>276750</v>
       </c>
       <c r="E9" t="n">
-        <v>266000</v>
+        <v>389500</v>
       </c>
       <c r="F9" t="n">
-        <v>163000</v>
+        <v>61000</v>
       </c>
       <c r="G9" t="n">
-        <v>25</v>
+        <v>15</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FY2023</t>
+          <t>FY2024</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>174000</v>
+        <v>207000</v>
       </c>
       <c r="D10" t="n">
-        <v>234900</v>
+        <v>279450</v>
       </c>
       <c r="E10" t="n">
-        <v>330600</v>
+        <v>393300</v>
       </c>
       <c r="F10" t="n">
-        <v>59000</v>
+        <v>125000</v>
       </c>
       <c r="G10" t="n">
-        <v>15</v>
+        <v>10</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FY2023</t>
+          <t>FY2024</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>205000</v>
+        <v>117000</v>
       </c>
       <c r="D11" t="n">
-        <v>276750</v>
+        <v>157950</v>
       </c>
       <c r="E11" t="n">
-        <v>389500</v>
+        <v>222300</v>
       </c>
       <c r="F11" t="n">
-        <v>61000</v>
+        <v>105000</v>
       </c>
       <c r="G11" t="n">
-        <v>15</v>
+        <v>25</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -3858,23 +4558,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>207000</v>
+        <v>197000</v>
       </c>
       <c r="D12" t="n">
-        <v>279450</v>
+        <v>265950</v>
       </c>
       <c r="E12" t="n">
-        <v>393300</v>
+        <v>374300</v>
       </c>
       <c r="F12" t="n">
-        <v>125000</v>
+        <v>83000</v>
       </c>
       <c r="G12" t="n">
-        <v>10</v>
+        <v>20</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -3885,24 +4590,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>117000</v>
+        <v>115000</v>
       </c>
       <c r="D13" t="n">
-        <v>157950</v>
+        <v>155250</v>
       </c>
       <c r="E13" t="n">
-        <v>222300</v>
+        <v>218500</v>
       </c>
       <c r="F13" t="n">
-        <v>105000</v>
+        <v>47000</v>
       </c>
       <c r="G13" t="n">
         <v>25</v>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3912,23 +4622,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>197000</v>
+        <v>206000</v>
       </c>
       <c r="D14" t="n">
-        <v>265950</v>
+        <v>278100</v>
       </c>
       <c r="E14" t="n">
-        <v>374300</v>
+        <v>391400</v>
       </c>
       <c r="F14" t="n">
-        <v>83000</v>
+        <v>29000</v>
       </c>
       <c r="G14" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -3939,24 +4654,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>115000</v>
+        <v>123000</v>
       </c>
       <c r="D15" t="n">
-        <v>155250</v>
+        <v>166050</v>
       </c>
       <c r="E15" t="n">
-        <v>218500</v>
+        <v>233700</v>
       </c>
       <c r="F15" t="n">
-        <v>47000</v>
+        <v>71000</v>
       </c>
       <c r="G15" t="n">
         <v>25</v>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3966,23 +4686,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>206000</v>
+        <v>139000</v>
       </c>
       <c r="D16" t="n">
-        <v>278100</v>
+        <v>187650</v>
       </c>
       <c r="E16" t="n">
-        <v>391400</v>
+        <v>264100</v>
       </c>
       <c r="F16" t="n">
-        <v>29000</v>
+        <v>98000</v>
       </c>
       <c r="G16" t="n">
-        <v>25</v>
+        <v>15</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -3993,7 +4718,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -4006,64 +4731,79 @@
         <v>233700</v>
       </c>
       <c r="F17" t="n">
-        <v>71000</v>
+        <v>26000</v>
       </c>
       <c r="G17" t="n">
-        <v>25</v>
+        <v>15</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2025</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>139000</v>
+        <v>146000</v>
       </c>
       <c r="D18" t="n">
-        <v>187650</v>
+        <v>197100</v>
       </c>
       <c r="E18" t="n">
-        <v>264100</v>
+        <v>277400</v>
       </c>
       <c r="F18" t="n">
-        <v>98000</v>
+        <v>104000</v>
       </c>
       <c r="G18" t="n">
-        <v>15</v>
+        <v>20</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2025</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>123000</v>
+        <v>205000</v>
       </c>
       <c r="D19" t="n">
-        <v>166050</v>
+        <v>276750</v>
       </c>
       <c r="E19" t="n">
-        <v>233700</v>
+        <v>389500</v>
       </c>
       <c r="F19" t="n">
-        <v>26000</v>
+        <v>37000</v>
       </c>
       <c r="G19" t="n">
-        <v>15</v>
+        <v>20</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -4074,23 +4814,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>146000</v>
+        <v>139000</v>
       </c>
       <c r="D20" t="n">
-        <v>197100</v>
+        <v>187650</v>
       </c>
       <c r="E20" t="n">
-        <v>277400</v>
+        <v>264100</v>
       </c>
       <c r="F20" t="n">
-        <v>104000</v>
+        <v>150000</v>
       </c>
       <c r="G20" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -4101,24 +4846,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>205000</v>
+        <v>181000</v>
       </c>
       <c r="D21" t="n">
-        <v>276750</v>
+        <v>244350</v>
       </c>
       <c r="E21" t="n">
-        <v>389500</v>
+        <v>343900</v>
       </c>
       <c r="F21" t="n">
-        <v>37000</v>
+        <v>157000</v>
       </c>
       <c r="G21" t="n">
         <v>20</v>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4128,23 +4878,28 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>139000</v>
+        <v>98000</v>
       </c>
       <c r="D22" t="n">
-        <v>187650</v>
+        <v>132300</v>
       </c>
       <c r="E22" t="n">
-        <v>264100</v>
+        <v>186200</v>
       </c>
       <c r="F22" t="n">
-        <v>150000</v>
+        <v>49000</v>
       </c>
       <c r="G22" t="n">
-        <v>25</v>
+        <v>20</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -4155,24 +4910,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>181000</v>
+        <v>117000</v>
       </c>
       <c r="D23" t="n">
-        <v>244350</v>
+        <v>157950</v>
       </c>
       <c r="E23" t="n">
-        <v>343900</v>
+        <v>222300</v>
       </c>
       <c r="F23" t="n">
-        <v>157000</v>
+        <v>168000</v>
       </c>
       <c r="G23" t="n">
         <v>20</v>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4182,23 +4942,28 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>98000</v>
+        <v>99000</v>
       </c>
       <c r="D24" t="n">
-        <v>132300</v>
+        <v>133650</v>
       </c>
       <c r="E24" t="n">
-        <v>186200</v>
+        <v>188100</v>
       </c>
       <c r="F24" t="n">
-        <v>49000</v>
+        <v>47000</v>
       </c>
       <c r="G24" t="n">
-        <v>20</v>
+        <v>30</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -4209,77 +4974,28 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>117000</v>
+        <v>150000</v>
       </c>
       <c r="D25" t="n">
-        <v>157950</v>
+        <v>202500</v>
       </c>
       <c r="E25" t="n">
-        <v>222300</v>
+        <v>285000</v>
       </c>
       <c r="F25" t="n">
-        <v>168000</v>
+        <v>108000</v>
       </c>
       <c r="G25" t="n">
         <v>20</v>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>FY2025</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Legal</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>99000</v>
-      </c>
-      <c r="D26" t="n">
-        <v>133650</v>
-      </c>
-      <c r="E26" t="n">
-        <v>188100</v>
-      </c>
-      <c r="F26" t="n">
-        <v>47000</v>
-      </c>
-      <c r="G26" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>FY2025</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D27" t="n">
-        <v>202500</v>
-      </c>
-      <c r="E27" t="n">
-        <v>285000</v>
-      </c>
-      <c r="F27" t="n">
-        <v>108000</v>
-      </c>
-      <c r="G27" t="n">
-        <v>20</v>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>SYNTHETIC - not real Apple data</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>